<commit_message>
updating knots, velocity is broken so it needs an updata
</commit_message>
<xml_diff>
--- a/knots/knoten_summary.xlsx
+++ b/knots/knoten_summary.xlsx
@@ -637,18 +637,18 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>39696.14439928731</v>
+        <v>41607.97871691309</v>
       </c>
       <c r="C2" t="n">
-        <v>14679.74376296387</v>
+        <v>15191.72272502771</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>617k</t>
+          <t>0k</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>616549.2380444827</v>
+        <v>0</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -661,94 +661,94 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>53558</v>
+        <v>54550</v>
       </c>
       <c r="I2" t="n">
-        <v>39696</v>
+        <v>41607</v>
       </c>
       <c r="J2" t="n">
-        <v>724</v>
+        <v>562</v>
       </c>
       <c r="K2" t="n">
-        <v>10480</v>
+        <v>7466</v>
       </c>
       <c r="L2" t="n">
-        <v>5080</v>
+        <v>7564</v>
       </c>
       <c r="M2" t="n">
-        <v>7808</v>
+        <v>9710</v>
       </c>
       <c r="N2" t="n">
-        <v>12888</v>
+        <v>17274</v>
       </c>
       <c r="O2" t="n">
-        <v>22512</v>
+        <v>23723</v>
       </c>
       <c r="P2" t="n">
-        <v>928483.5730743674</v>
+        <v>1302176.099319996</v>
       </c>
       <c r="Q2" t="n">
-        <v>732970.5933277697</v>
+        <v>1021729.230378219</v>
       </c>
       <c r="R2" t="n">
-        <v>15467.365093518</v>
+        <v>10176.82094013536</v>
       </c>
       <c r="S2" t="n">
-        <v>275601.3403391327</v>
+        <v>124677.5978033582</v>
       </c>
       <c r="T2" t="n">
-        <v>14412.72692327057</v>
+        <v>39031.85863212649</v>
       </c>
       <c r="U2" t="n">
-        <v>55552.19254083238</v>
+        <v>113319.7152334225</v>
       </c>
       <c r="V2" t="n">
-        <v>69964.91946410295</v>
+        <v>152351.5738655489</v>
       </c>
       <c r="W2" t="n">
-        <v>339416.9116879085</v>
+        <v>140968.3542028361</v>
       </c>
       <c r="X2" t="n">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="Y2" t="n">
-        <v>26.4</v>
+        <v>17.9</v>
       </c>
       <c r="Z2" t="n">
-        <v>12.8</v>
+        <v>18.2</v>
       </c>
       <c r="AA2" t="n">
-        <v>19.7</v>
+        <v>23.3</v>
       </c>
       <c r="AB2" t="n">
-        <v>32.5</v>
+        <v>41.5</v>
       </c>
       <c r="AC2" t="n">
-        <v>56.7</v>
+        <v>57</v>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>2%</t>
+          <t>1%</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>23%</t>
         </is>
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>42%</t>
         </is>
       </c>
       <c r="AI2" t="inlineStr">
@@ -757,19 +757,19 @@
         </is>
       </c>
       <c r="AJ2" t="n">
-        <v>320.8848640540263</v>
+        <v>336.3392288138488</v>
       </c>
       <c r="AK2" t="n">
-        <v>2184.299005304827</v>
+        <v>2289.498587316942</v>
       </c>
       <c r="AL2" t="n">
-        <v>2433.169174615234</v>
+        <v>2550.354770320143</v>
       </c>
       <c r="AM2" t="n">
         <v>10.2282312264523</v>
       </c>
       <c r="AN2" t="n">
-        <v>56.46055293447643</v>
+        <v>58.42970278856811</v>
       </c>
     </row>
     <row r="3">
@@ -779,18 +779,18 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>23018.21113144683</v>
+        <v>27434.17901233025</v>
       </c>
       <c r="C3" t="n">
-        <v>21992.84729922871</v>
+        <v>26739.05870420755</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>924k</t>
+          <t>0k</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>923699.5865676056</v>
+        <v>0</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -803,115 +803,115 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>36761</v>
+        <v>37251</v>
       </c>
       <c r="I3" t="n">
-        <v>23018</v>
+        <v>27434</v>
       </c>
       <c r="J3" t="n">
-        <v>1804</v>
+        <v>1610</v>
       </c>
       <c r="K3" t="n">
-        <v>9310</v>
+        <v>7857</v>
       </c>
       <c r="L3" t="n">
-        <v>2658</v>
+        <v>4842</v>
       </c>
       <c r="M3" t="n">
-        <v>7258</v>
+        <v>11610</v>
       </c>
       <c r="N3" t="n">
-        <v>9916</v>
+        <v>16452</v>
       </c>
       <c r="O3" t="n">
-        <v>16523</v>
+        <v>20465</v>
       </c>
       <c r="P3" t="n">
-        <v>480016.8020532717</v>
+        <v>685881.2255584287</v>
       </c>
       <c r="Q3" t="n">
-        <v>340950.2453581307</v>
+        <v>502179.0519804134</v>
       </c>
       <c r="R3" t="n">
-        <v>20262.18941630103</v>
+        <v>24227.40328216191</v>
       </c>
       <c r="S3" t="n">
-        <v>159273.3310332766</v>
+        <v>103757.0677616429</v>
       </c>
       <c r="T3" t="n">
-        <v>9023.552110116161</v>
+        <v>28382.20535496958</v>
       </c>
       <c r="U3" t="n">
-        <v>51528.70305387807</v>
+        <v>129377.9142370557</v>
       </c>
       <c r="V3" t="n">
-        <v>60552.25516399422</v>
+        <v>157760.1195920253</v>
       </c>
       <c r="W3" t="n">
-        <v>199955.37506405</v>
+        <v>118875.395564785</v>
       </c>
       <c r="X3" t="n">
-        <v>7.8</v>
+        <v>5.9</v>
       </c>
       <c r="Y3" t="n">
-        <v>40.4</v>
+        <v>28.6</v>
       </c>
       <c r="Z3" t="n">
-        <v>11.5</v>
+        <v>17.6</v>
       </c>
       <c r="AA3" t="n">
-        <v>31.5</v>
+        <v>42.3</v>
       </c>
       <c r="AB3" t="n">
-        <v>43.1</v>
+        <v>60</v>
       </c>
       <c r="AC3" t="n">
-        <v>71.8</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
         <is>
-          <t>12%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>42%</t>
         </is>
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>60%</t>
         </is>
       </c>
       <c r="AI3" t="inlineStr">
         <is>
-          <t>72%</t>
+          <t>75%</t>
         </is>
       </c>
       <c r="AJ3" t="n">
-        <v>856.2231169610694</v>
+        <v>1020.48669773101</v>
       </c>
       <c r="AK3" t="n">
-        <v>1525.612100697691</v>
+        <v>1818.295750043669</v>
       </c>
       <c r="AL3" t="n">
-        <v>1703.729772441428</v>
+        <v>2030.584709597149</v>
       </c>
       <c r="AM3" t="n">
-        <v>10.45457293902288</v>
+        <v>10.45457293902287</v>
       </c>
       <c r="AN3" t="n">
-        <v>84.58787422780271</v>
+        <v>102.8425334777214</v>
       </c>
     </row>
     <row r="4">
@@ -921,18 +921,18 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>24728.66281842267</v>
+        <v>31342.07780111492</v>
       </c>
       <c r="C4" t="n">
-        <v>20418.07089564238</v>
+        <v>24995.98223371203</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>858k</t>
+          <t>0k</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>857558.9776169799</v>
+        <v>0</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -941,70 +941,70 @@
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="n">
-        <v>36456</v>
+        <v>37287</v>
       </c>
       <c r="I4" t="n">
-        <v>24728</v>
+        <v>31342</v>
       </c>
       <c r="J4" t="n">
-        <v>510</v>
+        <v>680</v>
       </c>
       <c r="K4" t="n">
-        <v>6500</v>
+        <v>4831</v>
       </c>
       <c r="L4" t="n">
-        <v>3268</v>
+        <v>5532</v>
       </c>
       <c r="M4" t="n">
-        <v>5067</v>
+        <v>7887</v>
       </c>
       <c r="N4" t="n">
-        <v>8335</v>
+        <v>13419</v>
       </c>
       <c r="O4" t="n">
-        <v>14236</v>
+        <v>17346</v>
       </c>
       <c r="P4" t="n">
-        <v>682013.7551089261</v>
+        <v>941380.6453833126</v>
       </c>
       <c r="Q4" t="n">
-        <v>508766.5574869515</v>
+        <v>798947.4825964131</v>
       </c>
       <c r="R4" t="n">
-        <v>7268.717892209909</v>
+        <v>2736.170203693602</v>
       </c>
       <c r="S4" t="n">
-        <v>191871.505167108</v>
+        <v>70950.51873338391</v>
       </c>
       <c r="T4" t="n">
-        <v>11511.13844407699</v>
+        <v>28595.70008226805</v>
       </c>
       <c r="U4" t="n">
-        <v>36351.78351440241</v>
+        <v>79650.25478076504</v>
       </c>
       <c r="V4" t="n">
-        <v>47862.9219584794</v>
+        <v>108245.9548630331</v>
       </c>
       <c r="W4" t="n">
-        <v>236764.1392193035</v>
+        <v>79759.17366850402</v>
       </c>
       <c r="X4" t="n">
-        <v>2.1</v>
+        <v>2.2</v>
       </c>
       <c r="Y4" t="n">
-        <v>26.3</v>
+        <v>15.4</v>
       </c>
       <c r="Z4" t="n">
-        <v>13.2</v>
+        <v>17.7</v>
       </c>
       <c r="AA4" t="n">
-        <v>20.5</v>
+        <v>25.2</v>
       </c>
       <c r="AB4" t="n">
-        <v>33.7</v>
+        <v>42.8</v>
       </c>
       <c r="AC4" t="n">
-        <v>57.6</v>
+        <v>55.3</v>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
@@ -1013,43 +1013,43 @@
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>34%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>58%</t>
+          <t>55%</t>
         </is>
       </c>
       <c r="AJ4" t="n">
-        <v>178.9071901700588</v>
+        <v>226.753994531052</v>
       </c>
       <c r="AK4" t="n">
-        <v>1363.86864882996</v>
+        <v>1728.620654339801</v>
       </c>
       <c r="AL4" t="n">
-        <v>1645.515421829648</v>
+        <v>2085.590828449369</v>
       </c>
       <c r="AM4" t="n">
-        <v>17.1160214765125</v>
+        <v>17.11602147651248</v>
       </c>
       <c r="AN4" t="n">
-        <v>78.53104190631683</v>
+        <v>96.13839320658472</v>
       </c>
     </row>
     <row r="5">
@@ -1059,18 +1059,18 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>22940.07618698369</v>
+        <v>22856.64759730838</v>
       </c>
       <c r="C5" t="n">
-        <v>20659.37405913336</v>
+        <v>20171.11809029439</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>868k</t>
+          <t>0k</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>867693.710483601</v>
+        <v>0</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -1083,115 +1083,115 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>35121</v>
+        <v>35443</v>
       </c>
       <c r="I5" t="n">
-        <v>22940</v>
+        <v>22856</v>
       </c>
       <c r="J5" t="n">
-        <v>1076</v>
+        <v>1482</v>
       </c>
       <c r="K5" t="n">
-        <v>7810</v>
+        <v>4863</v>
       </c>
       <c r="L5" t="n">
-        <v>2880</v>
+        <v>4826</v>
       </c>
       <c r="M5" t="n">
-        <v>5229</v>
+        <v>7095</v>
       </c>
       <c r="N5" t="n">
-        <v>8110</v>
+        <v>11922</v>
       </c>
       <c r="O5" t="n">
-        <v>14115</v>
+        <v>14431</v>
       </c>
       <c r="P5" t="n">
-        <v>708501.7436950764</v>
+        <v>959147.779927663</v>
       </c>
       <c r="Q5" t="n">
-        <v>562329.598141136</v>
+        <v>696337.9653769468</v>
       </c>
       <c r="R5" t="n">
-        <v>22221.79525634902</v>
+        <v>6799.057983833345</v>
       </c>
       <c r="S5" t="n">
-        <v>247907.8642264297</v>
+        <v>109855.2011915182</v>
       </c>
       <c r="T5" t="n">
-        <v>8809.295681723241</v>
+        <v>25239.79625537203</v>
       </c>
       <c r="U5" t="n">
-        <v>38365.14872752003</v>
+        <v>78618.75073566922</v>
       </c>
       <c r="V5" t="n">
-        <v>47174.44440924328</v>
+        <v>103858.5469910413</v>
       </c>
       <c r="W5" t="n">
-        <v>284368.8550056009</v>
+        <v>137365.2490663716</v>
       </c>
       <c r="X5" t="n">
-        <v>4.7</v>
+        <v>6.5</v>
       </c>
       <c r="Y5" t="n">
-        <v>34</v>
+        <v>21.3</v>
       </c>
       <c r="Z5" t="n">
-        <v>12.6</v>
+        <v>21.1</v>
       </c>
       <c r="AA5" t="n">
-        <v>22.8</v>
+        <v>31</v>
       </c>
       <c r="AB5" t="n">
-        <v>35.4</v>
+        <v>52.2</v>
       </c>
       <c r="AC5" t="n">
-        <v>61.5</v>
+        <v>63.1</v>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>34%</t>
+          <t>21%</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>21%</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>23%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>35%</t>
+          <t>52%</t>
         </is>
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>62%</t>
+          <t>63%</t>
         </is>
       </c>
       <c r="AJ5" t="n">
-        <v>283.3549516846304</v>
+        <v>282.3244449067157</v>
       </c>
       <c r="AK5" t="n">
-        <v>1191.526232938433</v>
+        <v>1187.192884070499</v>
       </c>
       <c r="AL5" t="n">
-        <v>1368.879697627774</v>
+        <v>1363.901348747091</v>
       </c>
       <c r="AM5" t="n">
         <v>12.95610308171629</v>
       </c>
       <c r="AN5" t="n">
-        <v>79.45913099666676</v>
+        <v>77.58122342420918</v>
       </c>
     </row>
     <row r="6">
@@ -1201,18 +1201,18 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14072.63608042767</v>
+        <v>19187.19751280618</v>
       </c>
       <c r="C6" t="n">
-        <v>6771.747255493533</v>
+        <v>10219.28648645637</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>284k</t>
+          <t>0k</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>284413.3847307284</v>
+        <v>0</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1225,70 +1225,70 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>29989</v>
+        <v>30141</v>
       </c>
       <c r="I6" t="n">
-        <v>14072</v>
+        <v>19187</v>
       </c>
       <c r="J6" t="n">
-        <v>2204</v>
+        <v>2995</v>
       </c>
       <c r="K6" t="n">
-        <v>6999</v>
+        <v>7859</v>
       </c>
       <c r="L6" t="n">
-        <v>3960</v>
+        <v>6518</v>
       </c>
       <c r="M6" t="n">
-        <v>5455</v>
+        <v>8969</v>
       </c>
       <c r="N6" t="n">
-        <v>9416</v>
+        <v>15487</v>
       </c>
       <c r="O6" t="n">
-        <v>12537</v>
+        <v>17520</v>
       </c>
       <c r="P6" t="n">
-        <v>258833.3861855119</v>
+        <v>352485.3801249463</v>
       </c>
       <c r="Q6" t="n">
-        <v>158229.4919082475</v>
+        <v>249925.3099793589</v>
       </c>
       <c r="R6" t="n">
-        <v>16368.98341736242</v>
+        <v>12687.47750874855</v>
       </c>
       <c r="S6" t="n">
-        <v>99029.18149178999</v>
+        <v>61264.15785650934</v>
       </c>
       <c r="T6" t="n">
-        <v>12072.37785237037</v>
+        <v>33459.97646144359</v>
       </c>
       <c r="U6" t="n">
-        <v>36287.83559194708</v>
+        <v>87428.14458315994</v>
       </c>
       <c r="V6" t="n">
-        <v>48360.21344431745</v>
+        <v>120888.1210446035</v>
       </c>
       <c r="W6" t="n">
-        <v>125262.758995632</v>
+        <v>78840.38981647494</v>
       </c>
       <c r="X6" t="n">
-        <v>15.7</v>
+        <v>15.6</v>
       </c>
       <c r="Y6" t="n">
-        <v>49.7</v>
+        <v>41</v>
       </c>
       <c r="Z6" t="n">
-        <v>28.1</v>
+        <v>34</v>
       </c>
       <c r="AA6" t="n">
-        <v>38.8</v>
+        <v>46.7</v>
       </c>
       <c r="AB6" t="n">
-        <v>66.90000000000001</v>
+        <v>80.7</v>
       </c>
       <c r="AC6" t="n">
-        <v>89.09999999999999</v>
+        <v>91.3</v>
       </c>
       <c r="AD6" t="inlineStr">
         <is>
@@ -1297,43 +1297,43 @@
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>41%</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
         <is>
-          <t>28%</t>
+          <t>34%</t>
         </is>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>47%</t>
         </is>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>67%</t>
+          <t>81%</t>
         </is>
       </c>
       <c r="AI6" t="inlineStr">
         <is>
-          <t>89%</t>
+          <t>91%</t>
         </is>
       </c>
       <c r="AJ6" t="n">
-        <v>428.676877138483</v>
+        <v>584.4752798140333</v>
       </c>
       <c r="AK6" t="n">
-        <v>792.7035895731851</v>
+        <v>1080.803927233292</v>
       </c>
       <c r="AL6" t="n">
-        <v>942.1367734373938</v>
+        <v>1284.547134787546</v>
       </c>
       <c r="AM6" t="n">
-        <v>15.86109236761882</v>
+        <v>15.86109236761881</v>
       </c>
       <c r="AN6" t="n">
-        <v>26.04518175189821</v>
+        <v>39.3049480248322</v>
       </c>
     </row>
     <row r="7">
@@ -1343,18 +1343,18 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3922.723728024716</v>
+        <v>4852.673219919192</v>
       </c>
       <c r="C7" t="n">
-        <v>474.5598622471519</v>
+        <v>696.6869483318945</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>20k</t>
+          <t>0k</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>19931.51421438038</v>
+        <v>0</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1363,115 +1363,115 @@
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="n">
-        <v>6544</v>
+        <v>6610</v>
       </c>
       <c r="I7" t="n">
-        <v>3922</v>
+        <v>4852</v>
       </c>
       <c r="J7" t="n">
-        <v>326</v>
+        <v>427</v>
       </c>
       <c r="K7" t="n">
-        <v>1406</v>
+        <v>1378</v>
       </c>
       <c r="L7" t="n">
-        <v>1069</v>
+        <v>1718</v>
       </c>
       <c r="M7" t="n">
-        <v>958</v>
+        <v>1458</v>
       </c>
       <c r="N7" t="n">
-        <v>2028</v>
+        <v>3176</v>
       </c>
       <c r="O7" t="n">
-        <v>2796</v>
+        <v>3650</v>
       </c>
       <c r="P7" t="n">
-        <v>80137.00827640857</v>
+        <v>110005.0409218307</v>
       </c>
       <c r="Q7" t="n">
-        <v>60056.83186784154</v>
+        <v>87332.76429836091</v>
       </c>
       <c r="R7" t="n">
-        <v>2619.297330560946</v>
+        <v>1127.379769241547</v>
       </c>
       <c r="S7" t="n">
-        <v>24723.04142514066</v>
+        <v>9675.190129634393</v>
       </c>
       <c r="T7" t="n">
-        <v>3357.691148387046</v>
+        <v>8822.991126851841</v>
       </c>
       <c r="U7" t="n">
-        <v>6541.725408928671</v>
+        <v>16115.0736359102</v>
       </c>
       <c r="V7" t="n">
-        <v>9899.416557315719</v>
+        <v>24938.06476276204</v>
       </c>
       <c r="W7" t="n">
-        <v>31109.14153170755</v>
+        <v>12688.05470624534</v>
       </c>
       <c r="X7" t="n">
-        <v>8.300000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="Y7" t="n">
-        <v>35.8</v>
+        <v>28.4</v>
       </c>
       <c r="Z7" t="n">
-        <v>27.3</v>
+        <v>35.4</v>
       </c>
       <c r="AA7" t="n">
-        <v>24.4</v>
+        <v>30</v>
       </c>
       <c r="AB7" t="n">
-        <v>51.7</v>
+        <v>65.5</v>
       </c>
       <c r="AC7" t="n">
-        <v>71.3</v>
+        <v>75.2</v>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
-          <t>8%</t>
+          <t>9%</t>
         </is>
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>36%</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>52%</t>
+          <t>65%</t>
         </is>
       </c>
       <c r="AI7" t="inlineStr">
         <is>
-          <t>71%</t>
+          <t>75%</t>
         </is>
       </c>
       <c r="AJ7" t="n">
-        <v>132.2599011256628</v>
+        <v>146.9658244107009</v>
       </c>
       <c r="AK7" t="n">
-        <v>200.2987817038388</v>
+        <v>265.0586555740285</v>
       </c>
       <c r="AL7" t="n">
-        <v>314.6996218343609</v>
+        <v>389.3046090103539</v>
       </c>
       <c r="AM7" t="n">
-        <v>36.3523919932563</v>
+        <v>31.91484266065315</v>
       </c>
       <c r="AN7" t="n">
-        <v>1.825230239412123</v>
+        <v>2.679565185891902</v>
       </c>
     </row>
     <row r="8">
@@ -1481,18 +1481,18 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8519.367454717401</v>
+        <v>10784.61211892607</v>
       </c>
       <c r="C8" t="n">
-        <v>803.803921714381</v>
+        <v>1019.247502273883</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>34k</t>
+          <t>0k</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>33759.764712004</v>
+        <v>0</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -1501,115 +1501,115 @@
       </c>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="n">
-        <v>14795</v>
+        <v>14934</v>
       </c>
       <c r="I8" t="n">
-        <v>8519</v>
+        <v>10784</v>
       </c>
       <c r="J8" t="n">
-        <v>391</v>
+        <v>471</v>
       </c>
       <c r="K8" t="n">
-        <v>2389</v>
+        <v>1813</v>
       </c>
       <c r="L8" t="n">
-        <v>1990</v>
+        <v>2865</v>
       </c>
       <c r="M8" t="n">
-        <v>1734</v>
+        <v>2832</v>
       </c>
       <c r="N8" t="n">
-        <v>3724</v>
+        <v>5697</v>
       </c>
       <c r="O8" t="n">
-        <v>5755</v>
+        <v>7027</v>
       </c>
       <c r="P8" t="n">
-        <v>187167.1059416583</v>
+        <v>264643.0943179412</v>
       </c>
       <c r="Q8" t="n">
-        <v>137938.9642971887</v>
+        <v>220259.0466312289</v>
       </c>
       <c r="R8" t="n">
-        <v>2599.234129179709</v>
+        <v>1230.819034911819</v>
       </c>
       <c r="S8" t="n">
-        <v>58776.74244477192</v>
+        <v>20194.27550912667</v>
       </c>
       <c r="T8" t="n">
-        <v>5498.737375599922</v>
+        <v>13333.72093654935</v>
       </c>
       <c r="U8" t="n">
-        <v>12257.14962050569</v>
+        <v>28889.38759893795</v>
       </c>
       <c r="V8" t="n">
-        <v>17755.88699610561</v>
+        <v>42223.1085354873</v>
       </c>
       <c r="W8" t="n">
-        <v>75280.59246095373</v>
+        <v>22578.91313625585</v>
       </c>
       <c r="X8" t="n">
-        <v>4.6</v>
+        <v>4.4</v>
       </c>
       <c r="Y8" t="n">
-        <v>28</v>
+        <v>16.8</v>
       </c>
       <c r="Z8" t="n">
-        <v>23.4</v>
+        <v>26.6</v>
       </c>
       <c r="AA8" t="n">
-        <v>20.4</v>
+        <v>26.3</v>
       </c>
       <c r="AB8" t="n">
-        <v>43.7</v>
+        <v>52.8</v>
       </c>
       <c r="AC8" t="n">
-        <v>67.59999999999999</v>
+        <v>65.2</v>
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>4%</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>28%</t>
+          <t>17%</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
         <is>
-          <t>23%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>44%</t>
+          <t>53%</t>
         </is>
       </c>
       <c r="AI8" t="inlineStr">
         <is>
-          <t>68%</t>
+          <t>65%</t>
         </is>
       </c>
       <c r="AJ8" t="n">
-        <v>308.8650973556491</v>
+        <v>390.9903275988591</v>
       </c>
       <c r="AK8" t="n">
-        <v>569.649107343909</v>
+        <v>721.1151179064066</v>
       </c>
       <c r="AL8" t="n">
-        <v>668.3336047850707</v>
+        <v>846.03918447719</v>
       </c>
       <c r="AM8" t="n">
         <v>14.76575421834395</v>
       </c>
       <c r="AN8" t="n">
-        <v>3.091553545055311</v>
+        <v>3.920182701053396</v>
       </c>
     </row>
     <row r="9">
@@ -1619,18 +1619,18 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11997.43187535459</v>
+        <v>17755.43774447074</v>
       </c>
       <c r="C9" t="n">
-        <v>2217.813750579714</v>
+        <v>3331.478624297272</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>93k</t>
+          <t>0k</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>93148.17752434796</v>
+        <v>0</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1643,70 +1643,70 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>19853</v>
+        <v>20102</v>
       </c>
       <c r="I9" t="n">
-        <v>11997</v>
+        <v>17755</v>
       </c>
       <c r="J9" t="n">
-        <v>953</v>
+        <v>1473</v>
       </c>
       <c r="K9" t="n">
-        <v>3007</v>
+        <v>3563</v>
       </c>
       <c r="L9" t="n">
-        <v>2778</v>
+        <v>5394</v>
       </c>
       <c r="M9" t="n">
-        <v>3855</v>
+        <v>6291</v>
       </c>
       <c r="N9" t="n">
-        <v>6634</v>
+        <v>11685</v>
       </c>
       <c r="O9" t="n">
-        <v>8813</v>
+        <v>13707</v>
       </c>
       <c r="P9" t="n">
-        <v>180463.7415965202</v>
+        <v>259455.8686630169</v>
       </c>
       <c r="Q9" t="n">
-        <v>125062.286589499</v>
+        <v>233418.3542512017</v>
       </c>
       <c r="R9" t="n">
-        <v>7867.013365843048</v>
+        <v>4060.569875190444</v>
       </c>
       <c r="S9" t="n">
-        <v>46583.16239076383</v>
+        <v>13958.49986267905</v>
       </c>
       <c r="T9" t="n">
-        <v>7987.479061256501</v>
+        <v>24329.86076587313</v>
       </c>
       <c r="U9" t="n">
-        <v>24886.90103719667</v>
+        <v>63940.13960208505</v>
       </c>
       <c r="V9" t="n">
-        <v>32874.38009845317</v>
+        <v>88270.00036795819</v>
       </c>
       <c r="W9" t="n">
-        <v>76106.80887401954</v>
+        <v>17739.74654411246</v>
       </c>
       <c r="X9" t="n">
-        <v>7.9</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="Y9" t="n">
-        <v>25.1</v>
+        <v>20.1</v>
       </c>
       <c r="Z9" t="n">
-        <v>23.2</v>
+        <v>30.4</v>
       </c>
       <c r="AA9" t="n">
-        <v>32.1</v>
+        <v>35.4</v>
       </c>
       <c r="AB9" t="n">
-        <v>55.3</v>
+        <v>65.8</v>
       </c>
       <c r="AC9" t="n">
-        <v>73.5</v>
+        <v>77.2</v>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
@@ -1715,43 +1715,43 @@
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
         <is>
-          <t>23%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>35%</t>
         </is>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>66%</t>
         </is>
       </c>
       <c r="AI9" t="inlineStr">
         <is>
-          <t>73%</t>
+          <t>77%</t>
         </is>
       </c>
       <c r="AJ9" t="n">
-        <v>161.6681284482188</v>
+        <v>239.2585696463986</v>
       </c>
       <c r="AK9" t="n">
-        <v>711.5098998652848</v>
+        <v>1052.989494992177</v>
       </c>
       <c r="AL9" t="n">
-        <v>857.6744710813991</v>
+        <v>1269.303783886464</v>
       </c>
       <c r="AM9" t="n">
-        <v>17.04196360558835</v>
+        <v>17.04196360558834</v>
       </c>
       <c r="AN9" t="n">
-        <v>8.530052886845052</v>
+        <v>12.81337932422028</v>
       </c>
     </row>
     <row r="10">
@@ -1761,18 +1761,18 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>22147.42349938014</v>
+        <v>29636.54689183965</v>
       </c>
       <c r="C10" t="n">
-        <v>9098.479367486825</v>
+        <v>11433.37230360543</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>382k</t>
+          <t>0k</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>382136.1334344466</v>
+        <v>0</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -1781,70 +1781,70 @@
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="n">
-        <v>34378</v>
+        <v>35115</v>
       </c>
       <c r="I10" t="n">
-        <v>22147</v>
+        <v>29636</v>
       </c>
       <c r="J10" t="n">
-        <v>559</v>
+        <v>796</v>
       </c>
       <c r="K10" t="n">
-        <v>5233</v>
+        <v>4108</v>
       </c>
       <c r="L10" t="n">
-        <v>3661</v>
+        <v>6303</v>
       </c>
       <c r="M10" t="n">
-        <v>4759</v>
+        <v>7741</v>
       </c>
       <c r="N10" t="n">
-        <v>8421</v>
+        <v>14044</v>
       </c>
       <c r="O10" t="n">
-        <v>13003</v>
+        <v>17193</v>
       </c>
       <c r="P10" t="n">
-        <v>588090.875419133</v>
+        <v>808694.7829676548</v>
       </c>
       <c r="Q10" t="n">
-        <v>425132.3155284899</v>
+        <v>691160.0396348013</v>
       </c>
       <c r="R10" t="n">
-        <v>5311.417222279578</v>
+        <v>1799.008869458885</v>
       </c>
       <c r="S10" t="n">
-        <v>150282.6540850274</v>
+        <v>62796.36420637844</v>
       </c>
       <c r="T10" t="n">
-        <v>12728.27686431241</v>
+        <v>32541.08529075133</v>
       </c>
       <c r="U10" t="n">
-        <v>32539.30083359606</v>
+        <v>74095.01907207996</v>
       </c>
       <c r="V10" t="n">
-        <v>45267.57769790848</v>
+        <v>106636.1043628313</v>
       </c>
       <c r="W10" t="n">
-        <v>192148.5095911238</v>
+        <v>67821.71642717194</v>
       </c>
       <c r="X10" t="n">
-        <v>2.5</v>
+        <v>2.7</v>
       </c>
       <c r="Y10" t="n">
-        <v>23.6</v>
+        <v>13.9</v>
       </c>
       <c r="Z10" t="n">
-        <v>16.5</v>
+        <v>21.3</v>
       </c>
       <c r="AA10" t="n">
-        <v>21.5</v>
+        <v>26.1</v>
       </c>
       <c r="AB10" t="n">
-        <v>38</v>
+        <v>47.4</v>
       </c>
       <c r="AC10" t="n">
-        <v>58.7</v>
+        <v>58</v>
       </c>
       <c r="AD10" t="inlineStr">
         <is>
@@ -1853,43 +1853,43 @@
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
         <is>
-          <t>17%</t>
+          <t>21%</t>
         </is>
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>21%</t>
+          <t>26%</t>
         </is>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>47%</t>
         </is>
       </c>
       <c r="AI10" t="inlineStr">
         <is>
-          <t>59%</t>
+          <t>58%</t>
         </is>
       </c>
       <c r="AJ10" t="n">
-        <v>457.8088403681014</v>
+        <v>612.6163237655029</v>
       </c>
       <c r="AK10" t="n">
-        <v>1275.348876794453</v>
+        <v>1706.606494955574</v>
       </c>
       <c r="AL10" t="n">
-        <v>1506.436450746132</v>
+        <v>2015.836041305832</v>
       </c>
       <c r="AM10" t="n">
         <v>15.34001476379715</v>
       </c>
       <c r="AN10" t="n">
-        <v>34.99415141341087</v>
+        <v>43.9745088600209</v>
       </c>
     </row>
     <row r="11">
@@ -1899,18 +1899,18 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>32211.38573110382</v>
+        <v>30669.00722193616</v>
       </c>
       <c r="C11" t="n">
-        <v>10004.18283391663</v>
+        <v>9466.066394832513</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>420k</t>
+          <t>0k</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>420175.6790244986</v>
+        <v>0</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -1919,115 +1919,115 @@
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="n">
-        <v>47924</v>
+        <v>48571</v>
       </c>
       <c r="I11" t="n">
-        <v>32211</v>
+        <v>30669</v>
       </c>
       <c r="J11" t="n">
-        <v>1326</v>
+        <v>1033</v>
       </c>
       <c r="K11" t="n">
-        <v>9975</v>
+        <v>5876</v>
       </c>
       <c r="L11" t="n">
-        <v>2824</v>
+        <v>4121</v>
       </c>
       <c r="M11" t="n">
-        <v>5463</v>
+        <v>8312</v>
       </c>
       <c r="N11" t="n">
-        <v>8288</v>
+        <v>12433</v>
       </c>
       <c r="O11" t="n">
-        <v>17412</v>
+        <v>17106</v>
       </c>
       <c r="P11" t="n">
-        <v>959788.7531180301</v>
+        <v>1228182.760052689</v>
       </c>
       <c r="Q11" t="n">
-        <v>685458.1202146559</v>
+        <v>752095.8453728155</v>
       </c>
       <c r="R11" t="n">
-        <v>28566.93164612983</v>
+        <v>56482.56810188608</v>
       </c>
       <c r="S11" t="n">
-        <v>290881.7301165886</v>
+        <v>263487.8144171963</v>
       </c>
       <c r="T11" t="n">
-        <v>9917.807297500432</v>
+        <v>24620.97264656985</v>
       </c>
       <c r="U11" t="n">
-        <v>36389.04969604195</v>
+        <v>82338.19637278139</v>
       </c>
       <c r="V11" t="n">
-        <v>46306.85699354237</v>
+        <v>106959.1690193512</v>
       </c>
       <c r="W11" t="n">
-        <v>332158.7642355731</v>
+        <v>276353.2500717398</v>
       </c>
       <c r="X11" t="n">
-        <v>4.1</v>
+        <v>3.4</v>
       </c>
       <c r="Y11" t="n">
-        <v>31</v>
+        <v>19.2</v>
       </c>
       <c r="Z11" t="n">
-        <v>8.800000000000001</v>
+        <v>13.4</v>
       </c>
       <c r="AA11" t="n">
-        <v>17</v>
+        <v>27.1</v>
       </c>
       <c r="AB11" t="n">
-        <v>25.7</v>
+        <v>40.5</v>
       </c>
       <c r="AC11" t="n">
-        <v>54.1</v>
+        <v>55.8</v>
       </c>
       <c r="AD11" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>3%</t>
         </is>
       </c>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>19%</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>9%</t>
+          <t>13%</t>
         </is>
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>17%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>41%</t>
         </is>
       </c>
       <c r="AI11" t="inlineStr">
         <is>
-          <t>54%</t>
+          <t>56%</t>
         </is>
       </c>
       <c r="AJ11" t="n">
-        <v>336.4871731785852</v>
+        <v>320.3751502791765</v>
       </c>
       <c r="AK11" t="n">
-        <v>1694.612649533746</v>
+        <v>1613.469473831105</v>
       </c>
       <c r="AL11" t="n">
-        <v>2516.163393465926</v>
+        <v>2395.68188496973</v>
       </c>
       <c r="AM11" t="n">
-        <v>32.65092982695861</v>
+        <v>32.6509298269586</v>
       </c>
       <c r="AN11" t="n">
-        <v>38.47762628429474</v>
+        <v>36.40794767243274</v>
       </c>
     </row>
   </sheetData>

</xml_diff>